<commit_message>
issue fix for archive folder
</commit_message>
<xml_diff>
--- a/sampleData/Direct.xlsx
+++ b/sampleData/Direct.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vijaytomar/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vijaytomar/AZOnline_Automation/AZOnline/sampleData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{874D5089-A57F-E84C-92C8-AD13E0DAA5FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0795CEFD-2FA1-9E4C-A8E0-7909C0EED8E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-1480" yWindow="-21000" windowWidth="38400" windowHeight="21000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19960" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master_Template" sheetId="1" r:id="rId1"/>
@@ -13472,9 +13472,11 @@
   <dimension ref="A1:E893"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="5" width="18" customWidth="1"/>
+    <col min="1" max="1" width="24" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="34.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="37.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="30.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="38.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">

</xml_diff>